<commit_message>
Add temperature-conditioned D3 DO envelopes
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
   <si>
     <t>sensor_id</t>
   </si>
@@ -64,6 +64,15 @@
     <t>mean_soft_high_exceedance_rate</t>
   </si>
   <si>
+    <t>mean_soft_high_exceedance_rate_evaluable</t>
+  </si>
+  <si>
+    <t>temperature_upper_mean_coverage</t>
+  </si>
+  <si>
+    <t>soft_high_scored</t>
+  </si>
+  <si>
     <t>physical_low_window_rate</t>
   </si>
   <si>
@@ -169,7 +178,7 @@
     <t>soft_bound</t>
   </si>
   <si>
-    <t>v2.4.0</t>
+    <t>v2.5.0</t>
   </si>
 </sst>
 </file>
@@ -527,10 +536,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF15"/>
+  <dimension ref="A1:AI15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:32">
+    <row r="1" spans="1:35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -627,13 +636,22 @@
       <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" spans="1:35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C2">
         <v>3072</v>
@@ -648,90 +666,99 @@
         <v>0.9959147135416667</v>
       </c>
       <c r="G2">
-        <v>4.985275620044693</v>
+        <v>4.965563109983805</v>
       </c>
       <c r="H2">
         <v>5</v>
       </c>
       <c r="I2">
-        <v>3.361516881358067</v>
+        <v>3.179518045560728</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0.004575163398692811</v>
+        <v>0.02516339869281046</v>
       </c>
       <c r="L2">
-        <v>0.06470588235294118</v>
+        <v>0.05228758169934641</v>
       </c>
       <c r="M2">
         <v>0.004231770833333333</v>
       </c>
       <c r="N2">
-        <v>0.001953125</v>
+        <v>0.02571614583333333</v>
       </c>
       <c r="O2">
         <v>9.156512909776618E-05</v>
       </c>
       <c r="P2">
-        <v>0.0002529373368146214</v>
+        <v>0.008047758920800696</v>
       </c>
       <c r="Q2">
+        <v>0.008108626548284556</v>
+      </c>
+      <c r="R2">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="S2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T2">
         <v>0.004231770833333333</v>
       </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
       <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
         <v>0.003580729166666667</v>
       </c>
-      <c r="V2">
+      <c r="Y2">
         <v>0.06640625</v>
       </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
         <v>0.06640625</v>
       </c>
-      <c r="Y2">
+      <c r="AB2">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="Z2">
+      <c r="AC2">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AA2">
-        <v>0</v>
-      </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-      <c r="AC2">
-        <v>0.06928104575163399</v>
-      </c>
       <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0.07745098039215687</v>
+      </c>
+      <c r="AG2">
         <v>0.000326797385620915</v>
       </c>
-      <c r="AE2" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AH2" t="s">
         <v>51</v>
       </c>
+      <c r="AI2" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="3" spans="1:32">
+    <row r="3" spans="1:35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C3">
         <v>3072</v>
@@ -746,90 +773,99 @@
         <v>0.9959201388888889</v>
       </c>
       <c r="G3">
-        <v>4.971187985955314</v>
+        <v>4.934058033997839</v>
       </c>
       <c r="H3">
         <v>5</v>
       </c>
       <c r="I3">
-        <v>3.511698701960541</v>
+        <v>3.162855452053948</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0.001633986928104575</v>
+        <v>0.05849673202614379</v>
       </c>
       <c r="L3">
-        <v>0.1745098039215686</v>
+        <v>0.1418300653594771</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>0.001627604166666667</v>
+        <v>0.0615234375</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>0.0002338990426457789</v>
+        <v>0.01225794168842472</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>0.01235065219774197</v>
       </c>
       <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
+        <v>0.991742819843342</v>
+      </c>
+      <c r="S3" t="b">
+        <v>1</v>
       </c>
       <c r="T3">
         <v>0</v>
       </c>
       <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
         <v>0.00390625</v>
       </c>
-      <c r="V3">
+      <c r="Y3">
         <v>0.1754557291666667</v>
       </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
-      <c r="X3">
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
         <v>0.1754557291666667</v>
       </c>
-      <c r="Y3">
+      <c r="AB3">
         <v>0.0478515625</v>
       </c>
-      <c r="Z3">
+      <c r="AC3">
         <v>0.0009765625</v>
       </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
-      <c r="AC3">
-        <v>0.1761437908496732</v>
-      </c>
       <c r="AD3">
+        <v>0</v>
+      </c>
+      <c r="AE3">
+        <v>0</v>
+      </c>
+      <c r="AF3">
+        <v>0.2003267973856209</v>
+      </c>
+      <c r="AG3">
         <v>0.0009803921568627451</v>
       </c>
-      <c r="AE3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF3" t="s">
+      <c r="AH3" t="s">
         <v>51</v>
       </c>
+      <c r="AI3" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="4" spans="1:32">
+    <row r="4" spans="1:35">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>3072</v>
@@ -844,7 +880,7 @@
         <v>0.9959120008680556</v>
       </c>
       <c r="G4">
-        <v>4.960479215403539</v>
+        <v>4.960499375821997</v>
       </c>
       <c r="H4">
         <v>5</v>
@@ -856,78 +892,87 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0.000326797385620915</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>0.2532679738562091</v>
+        <v>0.2535947712418301</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>0.0003255208333333333</v>
+        <v>0.003255208333333333</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>8.159268929503916E-06</v>
+        <v>0.0009818320278503049</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>0.0009892579195440098</v>
       </c>
       <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="S4" t="b">
         <v>0</v>
       </c>
       <c r="T4">
         <v>0</v>
       </c>
       <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
         <v>0.0078125</v>
       </c>
-      <c r="V4">
+      <c r="Y4">
         <v>0.2526041666666667</v>
       </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
         <v>0.2526041666666667</v>
       </c>
-      <c r="Y4">
+      <c r="AB4">
         <v>0.0107421875</v>
       </c>
-      <c r="Z4">
+      <c r="AC4">
         <v>0.00390625</v>
       </c>
-      <c r="AA4">
-        <v>0</v>
-      </c>
-      <c r="AB4">
-        <v>0</v>
-      </c>
-      <c r="AC4">
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
         <v>0.2535947712418301</v>
       </c>
-      <c r="AD4">
+      <c r="AG4">
         <v>0.00392156862745098</v>
       </c>
-      <c r="AE4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF4" t="s">
+      <c r="AH4" t="s">
         <v>51</v>
       </c>
+      <c r="AI4" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="5" spans="1:32">
+    <row r="5" spans="1:35">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C5">
         <v>3072</v>
@@ -971,61 +1016,67 @@
       <c r="P5">
         <v>0</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5" t="b">
+        <v>0</v>
+      </c>
+      <c r="T5">
         <v>0.962890625</v>
       </c>
-      <c r="R5">
+      <c r="U5">
         <v>0.962890625</v>
       </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
         <v>0.0009765625</v>
       </c>
-      <c r="V5">
+      <c r="Y5">
         <v>0.004231770833333333</v>
       </c>
-      <c r="W5">
-        <v>0</v>
-      </c>
-      <c r="X5">
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
         <v>0.004231770833333333</v>
       </c>
-      <c r="Y5">
-        <v>0</v>
-      </c>
-      <c r="Z5">
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AA5">
-        <v>0</v>
-      </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
-      <c r="AC5">
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+      <c r="AF5">
         <v>0.004248366013071895</v>
       </c>
-      <c r="AD5">
+      <c r="AG5">
         <v>0.000326797385620915</v>
       </c>
-      <c r="AE5" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF5" t="s">
+      <c r="AH5" t="s">
         <v>51</v>
       </c>
+      <c r="AI5" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="6" spans="1:32">
+    <row r="6" spans="1:35">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C6">
         <v>3072</v>
@@ -1040,90 +1091,99 @@
         <v>0.9959092881944445</v>
       </c>
       <c r="G6">
-        <v>4.989948398719691</v>
+        <v>4.940850418673874</v>
       </c>
       <c r="H6">
         <v>5</v>
       </c>
       <c r="I6">
-        <v>4.039039148817691</v>
+        <v>3.241887004861091</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0.00326797385620915</v>
+        <v>0.0457516339869281</v>
       </c>
       <c r="L6">
-        <v>0.04771241830065359</v>
+        <v>0.04084967320261438</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>0.003580729166666667</v>
+        <v>0.04720052083333334</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0.0002610966057441253</v>
+        <v>0.01921030161411823</v>
       </c>
       <c r="Q6">
-        <v>0</v>
+        <v>0.01935559491800667</v>
       </c>
       <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
+        <v>0.991742819843342</v>
+      </c>
+      <c r="S6" t="b">
+        <v>1</v>
       </c>
       <c r="T6">
         <v>0</v>
       </c>
       <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
         <v>0.005208333333333333</v>
       </c>
-      <c r="V6">
+      <c r="Y6">
         <v>0.05078125</v>
       </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-      <c r="X6">
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
         <v>0.05078125</v>
       </c>
-      <c r="Y6">
+      <c r="AB6">
         <v>0.0009765625</v>
       </c>
-      <c r="Z6">
+      <c r="AC6">
         <v>0.001302083333333333</v>
       </c>
-      <c r="AA6">
-        <v>0</v>
-      </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-      <c r="AC6">
-        <v>0.05098039215686274</v>
-      </c>
       <c r="AD6">
+        <v>0</v>
+      </c>
+      <c r="AE6">
+        <v>0</v>
+      </c>
+      <c r="AF6">
+        <v>0.08660130718954248</v>
+      </c>
+      <c r="AG6">
         <v>0.00130718954248366</v>
       </c>
-      <c r="AE6" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF6" t="s">
+      <c r="AH6" t="s">
         <v>51</v>
       </c>
+      <c r="AI6" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" spans="1:35">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C7">
         <v>3072</v>
@@ -1138,90 +1198,99 @@
         <v>0.9959038628472223</v>
       </c>
       <c r="G7">
-        <v>4.998378256273359</v>
+        <v>4.957886397575694</v>
       </c>
       <c r="H7">
         <v>5</v>
       </c>
       <c r="I7">
-        <v>4.724365167861407</v>
+        <v>3.359895220673947</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>0.03790849673202614</v>
       </c>
       <c r="L7">
-        <v>0.01535947712418301</v>
+        <v>0.01339869281045752</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>0</v>
+        <v>0.03776041666666666</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>0.01685515263546672</v>
       </c>
       <c r="Q7">
-        <v>0</v>
+        <v>0.01698263323744493</v>
       </c>
       <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
+        <v>0.991742819843342</v>
+      </c>
+      <c r="S7" t="b">
+        <v>1</v>
       </c>
       <c r="T7">
         <v>0</v>
       </c>
       <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
         <v>0.0009765625</v>
       </c>
-      <c r="V7">
+      <c r="Y7">
         <v>0.01529947916666667</v>
       </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-      <c r="X7">
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
         <v>0.01529947916666667</v>
       </c>
-      <c r="Y7">
+      <c r="AB7">
         <v>0.001302083333333333</v>
       </c>
-      <c r="Z7">
+      <c r="AC7">
         <v>0.0009765625</v>
       </c>
-      <c r="AA7">
-        <v>0</v>
-      </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-      <c r="AC7">
-        <v>0.01535947712418301</v>
-      </c>
       <c r="AD7">
+        <v>0</v>
+      </c>
+      <c r="AE7">
+        <v>0</v>
+      </c>
+      <c r="AF7">
+        <v>0.05130718954248366</v>
+      </c>
+      <c r="AG7">
         <v>0.0009803921568627451</v>
       </c>
-      <c r="AE7" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF7" t="s">
+      <c r="AH7" t="s">
         <v>51</v>
       </c>
+      <c r="AI7" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" spans="1:35">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C8">
         <v>3072</v>
@@ -1236,90 +1305,99 @@
         <v>0.9959364149305556</v>
       </c>
       <c r="G8">
-        <v>4.725489080903173</v>
+        <v>4.727035904034575</v>
       </c>
       <c r="H8">
         <v>4.724365167861407</v>
       </c>
       <c r="I8">
-        <v>3.232710494604983</v>
+        <v>4.43018736894732</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>0.00326797385620915</v>
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>0.7506535947712418</v>
+        <v>0.753921568627451</v>
       </c>
       <c r="M8">
         <v>0</v>
       </c>
       <c r="N8">
-        <v>0.004557291666666667</v>
+        <v>0.5335286458333334</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>0.0004270017406440383</v>
+        <v>0.08725617790361966</v>
       </c>
       <c r="Q8">
-        <v>0</v>
+        <v>0.08791612268881638</v>
       </c>
       <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8">
+        <v>0.991742796988247</v>
+      </c>
+      <c r="S8" t="b">
         <v>0</v>
       </c>
       <c r="T8">
         <v>0</v>
       </c>
       <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
         <v>0.263671875</v>
       </c>
-      <c r="V8">
+      <c r="Y8">
         <v>0.7509765625</v>
       </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
         <v>0.7509765625</v>
       </c>
-      <c r="Y8">
+      <c r="AB8">
         <v>0.3746744791666667</v>
       </c>
-      <c r="Z8">
+      <c r="AC8">
         <v>0.06966145833333333</v>
       </c>
-      <c r="AA8">
-        <v>0</v>
-      </c>
-      <c r="AB8">
-        <v>0</v>
-      </c>
-      <c r="AC8">
+      <c r="AD8">
+        <v>0</v>
+      </c>
+      <c r="AE8">
+        <v>0</v>
+      </c>
+      <c r="AF8">
         <v>0.753921568627451</v>
       </c>
-      <c r="AD8">
+      <c r="AG8">
         <v>0.06993464052287582</v>
       </c>
-      <c r="AE8" t="s">
+      <c r="AH8" t="s">
+        <v>52</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:35">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
         <v>49</v>
-      </c>
-      <c r="AF8" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>46</v>
       </c>
       <c r="C9">
         <v>3072</v>
@@ -1363,61 +1441,67 @@
       <c r="P9">
         <v>0</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9" t="b">
+        <v>0</v>
+      </c>
+      <c r="T9">
         <v>0.001627604166666667</v>
       </c>
-      <c r="R9">
+      <c r="U9">
         <v>0.001627604166666667</v>
       </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-      <c r="T9">
-        <v>0</v>
-      </c>
-      <c r="U9">
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
         <v>0.01009114583333333</v>
       </c>
-      <c r="V9">
+      <c r="Y9">
         <v>0.02864583333333333</v>
       </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-      <c r="X9">
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
         <v>0.02864583333333333</v>
       </c>
-      <c r="Y9">
+      <c r="AB9">
         <v>0.06673177083333333</v>
       </c>
-      <c r="Z9">
+      <c r="AC9">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AA9">
-        <v>0</v>
-      </c>
-      <c r="AB9">
-        <v>0</v>
-      </c>
-      <c r="AC9">
+      <c r="AD9">
+        <v>0</v>
+      </c>
+      <c r="AE9">
+        <v>0</v>
+      </c>
+      <c r="AF9">
         <v>0.02875816993464052</v>
       </c>
-      <c r="AD9">
+      <c r="AG9">
         <v>0.000326797385620915</v>
       </c>
-      <c r="AE9" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF9" t="s">
+      <c r="AH9" t="s">
         <v>51</v>
       </c>
+      <c r="AI9" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" spans="1:35">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C10">
         <v>3072</v>
@@ -1465,57 +1549,66 @@
         <v>0</v>
       </c>
       <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
       </c>
       <c r="T10">
         <v>0</v>
       </c>
       <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
         <v>0.0006510416666666666</v>
       </c>
-      <c r="V10">
+      <c r="Y10">
         <v>0.0009765625</v>
       </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-      <c r="X10">
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
         <v>0.0009765625</v>
       </c>
-      <c r="Y10">
-        <v>0</v>
-      </c>
-      <c r="Z10">
-        <v>0</v>
-      </c>
-      <c r="AA10">
-        <v>0</v>
-      </c>
       <c r="AB10">
         <v>0</v>
       </c>
       <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
+      </c>
+      <c r="AF10">
         <v>0.0009803921568627451</v>
       </c>
-      <c r="AD10">
-        <v>0</v>
-      </c>
-      <c r="AE10" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF10" t="s">
+      <c r="AG10">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="s">
         <v>51</v>
       </c>
+      <c r="AI10" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="11" spans="1:32">
+    <row r="11" spans="1:35">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C11">
         <v>3072</v>
@@ -1560,60 +1653,69 @@
         <v>0</v>
       </c>
       <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>1</v>
+      </c>
+      <c r="S11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11">
         <v>0.02278645833333333</v>
       </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-      <c r="T11">
-        <v>0</v>
-      </c>
       <c r="U11">
         <v>0</v>
       </c>
       <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
         <v>0.01009114583333333</v>
       </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-      <c r="X11">
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
         <v>0.01009114583333333</v>
       </c>
-      <c r="Y11">
-        <v>0</v>
-      </c>
-      <c r="Z11">
-        <v>0</v>
-      </c>
-      <c r="AA11">
-        <v>0</v>
-      </c>
       <c r="AB11">
         <v>0</v>
       </c>
       <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>0</v>
+      </c>
+      <c r="AF11">
         <v>0.03169934640522876</v>
       </c>
-      <c r="AD11">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF11" t="s">
+      <c r="AG11">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="s">
         <v>51</v>
       </c>
+      <c r="AI11" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="12" spans="1:32">
+    <row r="12" spans="1:35">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C12">
         <v>3072</v>
@@ -1658,60 +1760,69 @@
         <v>0</v>
       </c>
       <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>1</v>
+      </c>
+      <c r="S12" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12">
         <v>0.1848958333333333</v>
       </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-      <c r="T12">
-        <v>0</v>
-      </c>
       <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
         <v>0.06315104166666667</v>
       </c>
-      <c r="V12">
+      <c r="Y12">
         <v>0.2298177083333333</v>
       </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12">
+      <c r="Z12">
+        <v>0</v>
+      </c>
+      <c r="AA12">
         <v>0.2298177083333333</v>
       </c>
-      <c r="Y12">
+      <c r="AB12">
         <v>0.01106770833333333</v>
       </c>
-      <c r="Z12">
+      <c r="AC12">
         <v>0.008138020833333334</v>
       </c>
-      <c r="AA12">
+      <c r="AD12">
         <v>0.008823529411764706</v>
       </c>
-      <c r="AB12">
-        <v>0</v>
-      </c>
-      <c r="AC12">
+      <c r="AE12">
+        <v>0</v>
+      </c>
+      <c r="AF12">
         <v>0.369281045751634</v>
       </c>
-      <c r="AD12">
+      <c r="AG12">
         <v>0.008169934640522876</v>
       </c>
-      <c r="AE12" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF12" t="s">
+      <c r="AH12" t="s">
         <v>51</v>
       </c>
+      <c r="AI12" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="13" spans="1:32">
+    <row r="13" spans="1:35">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C13">
         <v>3072</v>
@@ -1759,57 +1870,66 @@
         <v>0</v>
       </c>
       <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="S13" t="b">
+        <v>1</v>
       </c>
       <c r="T13">
         <v>0</v>
       </c>
       <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
         <v>0.0009765625</v>
       </c>
-      <c r="V13">
+      <c r="Y13">
         <v>0.003255208333333333</v>
       </c>
-      <c r="W13">
-        <v>0</v>
-      </c>
-      <c r="X13">
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
         <v>0.003255208333333333</v>
       </c>
-      <c r="Y13">
-        <v>0</v>
-      </c>
-      <c r="Z13">
-        <v>0</v>
-      </c>
-      <c r="AA13">
-        <v>0</v>
-      </c>
       <c r="AB13">
         <v>0</v>
       </c>
       <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <v>0</v>
+      </c>
+      <c r="AF13">
         <v>0.00326797385620915</v>
       </c>
-      <c r="AD13">
-        <v>0</v>
-      </c>
-      <c r="AE13" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF13" t="s">
+      <c r="AG13">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="s">
         <v>51</v>
       </c>
+      <c r="AI13" t="s">
+        <v>54</v>
+      </c>
     </row>
-    <row r="14" spans="1:32">
+    <row r="14" spans="1:35">
       <c r="A14" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C14">
         <v>3072</v>
@@ -1854,17 +1974,17 @@
         <v>0</v>
       </c>
       <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>1</v>
+      </c>
+      <c r="S14" t="b">
+        <v>1</v>
+      </c>
+      <c r="T14">
         <v>0.002604166666666667</v>
       </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-      <c r="T14">
-        <v>0</v>
-      </c>
       <c r="U14">
         <v>0</v>
       </c>
@@ -1878,36 +1998,45 @@
         <v>0</v>
       </c>
       <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="Z14">
-        <v>0</v>
-      </c>
-      <c r="AA14">
-        <v>0</v>
-      </c>
-      <c r="AB14">
-        <v>0</v>
-      </c>
       <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
+      </c>
+      <c r="AF14">
         <v>0.00261437908496732</v>
       </c>
-      <c r="AD14">
-        <v>0</v>
-      </c>
-      <c r="AE14" t="s">
+      <c r="AG14">
+        <v>0</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>51</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35">
+      <c r="A15" t="s">
         <v>48</v>
       </c>
-      <c r="AF14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:32">
-      <c r="A15" t="s">
-        <v>45</v>
-      </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C15">
         <v>3072</v>
@@ -1952,52 +2081,61 @@
         <v>0</v>
       </c>
       <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>1</v>
+      </c>
+      <c r="S15" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15">
         <v>0.7119140625</v>
       </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-      <c r="T15">
-        <v>0</v>
-      </c>
       <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
         <v>0.1103515625</v>
       </c>
-      <c r="V15">
+      <c r="Y15">
         <v>0.2242838541666667</v>
       </c>
-      <c r="W15">
-        <v>0</v>
-      </c>
-      <c r="X15">
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
         <v>0.2242838541666667</v>
       </c>
-      <c r="Y15">
+      <c r="AB15">
         <v>0.1373697916666667</v>
       </c>
-      <c r="Z15">
+      <c r="AC15">
         <v>0.01204427083333333</v>
       </c>
-      <c r="AA15">
-        <v>0</v>
-      </c>
-      <c r="AB15">
-        <v>0</v>
-      </c>
-      <c r="AC15">
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
+        <v>0</v>
+      </c>
+      <c r="AF15">
         <v>0.8320261437908497</v>
       </c>
-      <c r="AD15">
+      <c r="AG15">
         <v>0.01209150326797386</v>
       </c>
-      <c r="AE15" t="s">
-        <v>50</v>
-      </c>
-      <c r="AF15" t="s">
-        <v>51</v>
+      <c r="AH15" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Align D3 temperature envelopes to minute scoring
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
@@ -178,7 +178,7 @@
     <t>soft_bound</t>
   </si>
   <si>
-    <t>v2.5.0</t>
+    <t>v2.6.0</t>
   </si>
 </sst>
 </file>
@@ -666,7 +666,7 @@
         <v>0.9959147135416667</v>
       </c>
       <c r="G2">
-        <v>4.965563109983805</v>
+        <v>4.964900060366542</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -678,25 +678,25 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0.02516339869281046</v>
+        <v>0.02647058823529412</v>
       </c>
       <c r="L2">
-        <v>0.05228758169934641</v>
+        <v>0.05163398692810457</v>
       </c>
       <c r="M2">
         <v>0.004231770833333333</v>
       </c>
       <c r="N2">
-        <v>0.02571614583333333</v>
+        <v>0.02766927083333333</v>
       </c>
       <c r="O2">
         <v>9.156512909776618E-05</v>
       </c>
       <c r="P2">
-        <v>0.008047758920800696</v>
+        <v>0.008297976501305485</v>
       </c>
       <c r="Q2">
-        <v>0.008108626548284556</v>
+        <v>0.008360736599802698</v>
       </c>
       <c r="R2">
         <v>0.991742819843342</v>
@@ -741,7 +741,7 @@
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>0.07745098039215687</v>
+        <v>0.07810457516339869</v>
       </c>
       <c r="AG2">
         <v>0.000326797385620915</v>
@@ -773,37 +773,37 @@
         <v>0.9959201388888889</v>
       </c>
       <c r="G3">
-        <v>4.934058033997839</v>
+        <v>4.932095428002538</v>
       </c>
       <c r="H3">
         <v>5</v>
       </c>
       <c r="I3">
-        <v>3.162855452053948</v>
+        <v>3.161787143765561</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0.05849673202614379</v>
+        <v>0.06372549019607843</v>
       </c>
       <c r="L3">
-        <v>0.1418300653594771</v>
+        <v>0.1405228758169935</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>0.0615234375</v>
+        <v>0.06673177083333333</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>0.01225794168842472</v>
+        <v>0.01285628807658834</v>
       </c>
       <c r="Q3">
-        <v>0.01235065219774197</v>
+        <v>0.01295352406006796</v>
       </c>
       <c r="R3">
         <v>0.991742819843342</v>
@@ -848,7 +848,7 @@
         <v>0</v>
       </c>
       <c r="AF3">
-        <v>0.2003267973856209</v>
+        <v>0.2042483660130719</v>
       </c>
       <c r="AG3">
         <v>0.0009803921568627451</v>
@@ -901,16 +901,16 @@
         <v>0</v>
       </c>
       <c r="N4">
-        <v>0.003255208333333333</v>
+        <v>0.0029296875</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>0.0009818320278503049</v>
+        <v>0.0007968885987815492</v>
       </c>
       <c r="Q4">
-        <v>0.0009892579195440098</v>
+        <v>0.0008029157075523404</v>
       </c>
       <c r="R4">
         <v>0.991742819843342</v>
@@ -1091,7 +1091,7 @@
         <v>0.9959092881944445</v>
       </c>
       <c r="G6">
-        <v>4.940850418673874</v>
+        <v>4.936918875966986</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -1103,25 +1103,25 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0.0457516339869281</v>
+        <v>0.05032679738562092</v>
       </c>
       <c r="L6">
-        <v>0.04084967320261438</v>
+        <v>0.03888888888888889</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>0.04720052083333334</v>
+        <v>0.05110677083333334</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>0.01921030161411823</v>
+        <v>0.02062729465154208</v>
       </c>
       <c r="Q6">
-        <v>0.01935559491800667</v>
+        <v>0.02078330510106048</v>
       </c>
       <c r="R6">
         <v>0.991742819843342</v>
@@ -1166,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="AF6">
-        <v>0.08660130718954248</v>
+        <v>0.08921568627450981</v>
       </c>
       <c r="AG6">
         <v>0.00130718954248366</v>
@@ -1198,7 +1198,7 @@
         <v>0.9959038628472223</v>
       </c>
       <c r="G7">
-        <v>4.957886397575694</v>
+        <v>4.957126307985793</v>
       </c>
       <c r="H7">
         <v>5</v>
@@ -1210,7 +1210,7 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0.03790849673202614</v>
+        <v>0.03856209150326798</v>
       </c>
       <c r="L7">
         <v>0.01339869281045752</v>
@@ -1219,16 +1219,16 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>0.03776041666666666</v>
+        <v>0.03841145833333334</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>0.01685515263546672</v>
+        <v>0.01709993070335184</v>
       </c>
       <c r="Q7">
-        <v>0.01698263323744493</v>
+        <v>0.0172292626356692</v>
       </c>
       <c r="R7">
         <v>0.991742819843342</v>
@@ -1273,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="AF7">
-        <v>0.05130718954248366</v>
+        <v>0.05196078431372549</v>
       </c>
       <c r="AG7">
         <v>0.0009803921568627451</v>
@@ -1326,16 +1326,16 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>0.5335286458333334</v>
+        <v>0.4508463541666667</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>0.08725617790361966</v>
+        <v>0.05474846459088568</v>
       </c>
       <c r="Q8">
-        <v>0.08791612268881638</v>
+        <v>0.0551625437377421</v>
       </c>
       <c r="R8">
         <v>0.991742796988247</v>

</xml_diff>

<commit_message>
Finalize D3 denominator semantics and publication figures
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
+++ b/Project 1 Data Quality Assessment/D3 Physical rationality and rate constraints/outputs/data/D3_sensor_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="56">
   <si>
     <t>sensor_id</t>
   </si>
@@ -70,6 +70,9 @@
     <t>temperature_upper_mean_coverage</t>
   </si>
   <si>
+    <t>soft_state_mean_determinable_fraction</t>
+  </si>
+  <si>
     <t>soft_high_scored</t>
   </si>
   <si>
@@ -178,7 +181,7 @@
     <t>soft_bound</t>
   </si>
   <si>
-    <t>v2.6.0</t>
+    <t>v2.7.0</t>
   </si>
 </sst>
 </file>
@@ -536,10 +539,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AI15"/>
+  <dimension ref="A1:AJ15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:35">
+    <row r="1" spans="1:36">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -645,28 +648,31 @@
       <c r="AI1" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
     </row>
-    <row r="2" spans="1:35">
+    <row r="2" spans="1:36">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C2">
         <v>3072</v>
       </c>
       <c r="D2">
-        <v>3060</v>
+        <v>3037</v>
       </c>
       <c r="E2">
-        <v>0.99609375</v>
+        <v>0.9886067708333334</v>
       </c>
       <c r="F2">
         <v>0.9959147135416667</v>
       </c>
       <c r="G2">
-        <v>4.964900060366542</v>
+        <v>4.964634239289305</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -678,10 +684,10 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>0.02647058823529412</v>
+        <v>0.02667105696410932</v>
       </c>
       <c r="L2">
-        <v>0.05163398692810457</v>
+        <v>0.05202502469542312</v>
       </c>
       <c r="M2">
         <v>0.004231770833333333</v>
@@ -701,15 +707,15 @@
       <c r="R2">
         <v>0.991742819843342</v>
       </c>
-      <c r="S2" t="b">
-        <v>1</v>
-      </c>
-      <c r="T2">
+      <c r="S2">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="T2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2">
         <v>0.004231770833333333</v>
       </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
       <c r="V2">
         <v>0</v>
       </c>
@@ -717,63 +723,66 @@
         <v>0</v>
       </c>
       <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
         <v>0.003580729166666667</v>
       </c>
-      <c r="Y2">
+      <c r="Z2">
         <v>0.06640625</v>
       </c>
-      <c r="Z2">
-        <v>0</v>
-      </c>
       <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
         <v>0.06640625</v>
-      </c>
-      <c r="AB2">
-        <v>0.0003255208333333333</v>
       </c>
       <c r="AC2">
         <v>0.0003255208333333333</v>
       </c>
       <c r="AD2">
-        <v>0</v>
+        <v>0.0003255208333333333</v>
       </c>
       <c r="AE2">
         <v>0</v>
       </c>
       <c r="AF2">
-        <v>0.07810457516339869</v>
+        <v>0</v>
       </c>
       <c r="AG2">
-        <v>0.000326797385620915</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>51</v>
+        <v>0.07869608165953243</v>
+      </c>
+      <c r="AH2">
+        <v>0.0003292723081988805</v>
       </c>
       <c r="AI2" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:35">
+    <row r="3" spans="1:36">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3">
         <v>3072</v>
       </c>
       <c r="D3">
-        <v>3060</v>
+        <v>3037</v>
       </c>
       <c r="E3">
-        <v>0.99609375</v>
+        <v>0.9886067708333334</v>
       </c>
       <c r="F3">
         <v>0.9959201388888889</v>
       </c>
       <c r="G3">
-        <v>4.932095428002538</v>
+        <v>4.93178496289583</v>
       </c>
       <c r="H3">
         <v>5</v>
@@ -785,10 +794,10 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>0.06372549019607843</v>
+        <v>0.0642081000987817</v>
       </c>
       <c r="L3">
-        <v>0.1405228758169935</v>
+        <v>0.1402700032927231</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -808,11 +817,11 @@
       <c r="R3">
         <v>0.991742819843342</v>
       </c>
-      <c r="S3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3">
-        <v>0</v>
+      <c r="S3">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="T3" t="b">
+        <v>1</v>
       </c>
       <c r="U3">
         <v>0</v>
@@ -824,48 +833,51 @@
         <v>0</v>
       </c>
       <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
         <v>0.00390625</v>
       </c>
-      <c r="Y3">
+      <c r="Z3">
         <v>0.1754557291666667</v>
       </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
       <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
         <v>0.1754557291666667</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>0.0478515625</v>
       </c>
-      <c r="AC3">
+      <c r="AD3">
         <v>0.0009765625</v>
       </c>
-      <c r="AD3">
-        <v>0</v>
-      </c>
       <c r="AE3">
         <v>0</v>
       </c>
       <c r="AF3">
-        <v>0.2042483660130719</v>
+        <v>0</v>
       </c>
       <c r="AG3">
-        <v>0.0009803921568627451</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>51</v>
+        <v>0.2044781033915048</v>
+      </c>
+      <c r="AH3">
+        <v>0.0009878169245966415</v>
       </c>
       <c r="AI3" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:35">
+    <row r="4" spans="1:36">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4">
         <v>3072</v>
@@ -915,10 +927,10 @@
       <c r="R4">
         <v>0.991742819843342</v>
       </c>
-      <c r="S4" t="b">
-        <v>0</v>
-      </c>
-      <c r="T4">
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4" t="b">
         <v>0</v>
       </c>
       <c r="U4">
@@ -931,48 +943,51 @@
         <v>0</v>
       </c>
       <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
         <v>0.0078125</v>
       </c>
-      <c r="Y4">
+      <c r="Z4">
         <v>0.2526041666666667</v>
       </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
       <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
         <v>0.2526041666666667</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
         <v>0.0107421875</v>
       </c>
-      <c r="AC4">
+      <c r="AD4">
         <v>0.00390625</v>
       </c>
-      <c r="AD4">
-        <v>0</v>
-      </c>
       <c r="AE4">
         <v>0</v>
       </c>
       <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
         <v>0.2535947712418301</v>
       </c>
-      <c r="AG4">
+      <c r="AH4">
         <v>0.00392156862745098</v>
       </c>
-      <c r="AH4" t="s">
-        <v>51</v>
-      </c>
       <c r="AI4" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:35">
+    <row r="5" spans="1:36">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C5">
         <v>3072</v>
@@ -1019,79 +1034,82 @@
       <c r="R5">
         <v>0</v>
       </c>
-      <c r="S5" t="b">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>0.962890625</v>
+      <c r="S5">
+        <v>1</v>
+      </c>
+      <c r="T5" t="b">
+        <v>0</v>
       </c>
       <c r="U5">
         <v>0.962890625</v>
       </c>
       <c r="V5">
-        <v>0</v>
+        <v>0.962890625</v>
       </c>
       <c r="W5">
         <v>0</v>
       </c>
       <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
         <v>0.0009765625</v>
       </c>
-      <c r="Y5">
+      <c r="Z5">
         <v>0.004231770833333333</v>
       </c>
-      <c r="Z5">
-        <v>0</v>
-      </c>
       <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
         <v>0.004231770833333333</v>
       </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
       <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AD5">
-        <v>0</v>
-      </c>
       <c r="AE5">
         <v>0</v>
       </c>
       <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
         <v>0.004248366013071895</v>
       </c>
-      <c r="AG5">
+      <c r="AH5">
         <v>0.000326797385620915</v>
       </c>
-      <c r="AH5" t="s">
-        <v>51</v>
-      </c>
       <c r="AI5" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:35">
+    <row r="6" spans="1:36">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6">
         <v>3072</v>
       </c>
       <c r="D6">
-        <v>3060</v>
+        <v>3037</v>
       </c>
       <c r="E6">
-        <v>0.99609375</v>
+        <v>0.9886067708333334</v>
       </c>
       <c r="F6">
         <v>0.9959092881944445</v>
       </c>
       <c r="G6">
-        <v>4.936918875966986</v>
+        <v>4.93648979343922</v>
       </c>
       <c r="H6">
         <v>5</v>
@@ -1103,10 +1121,10 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>0.05032679738562092</v>
+        <v>0.05070793546262759</v>
       </c>
       <c r="L6">
-        <v>0.03888888888888889</v>
+        <v>0.0388541323674679</v>
       </c>
       <c r="M6">
         <v>0</v>
@@ -1126,11 +1144,11 @@
       <c r="R6">
         <v>0.991742819843342</v>
       </c>
-      <c r="S6" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
+      <c r="S6">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="T6" t="b">
+        <v>1</v>
       </c>
       <c r="U6">
         <v>0</v>
@@ -1142,63 +1160,66 @@
         <v>0</v>
       </c>
       <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
         <v>0.005208333333333333</v>
       </c>
-      <c r="Y6">
+      <c r="Z6">
         <v>0.05078125</v>
       </c>
-      <c r="Z6">
-        <v>0</v>
-      </c>
       <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
         <v>0.05078125</v>
       </c>
-      <c r="AB6">
+      <c r="AC6">
         <v>0.0009765625</v>
       </c>
-      <c r="AC6">
+      <c r="AD6">
         <v>0.001302083333333333</v>
       </c>
-      <c r="AD6">
-        <v>0</v>
-      </c>
       <c r="AE6">
         <v>0</v>
       </c>
       <c r="AF6">
-        <v>0.08921568627450981</v>
+        <v>0</v>
       </c>
       <c r="AG6">
-        <v>0.00130718954248366</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>51</v>
+        <v>0.08956206783009549</v>
+      </c>
+      <c r="AH6">
+        <v>0.001317089232795522</v>
       </c>
       <c r="AI6" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:35">
+    <row r="7" spans="1:36">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C7">
         <v>3072</v>
       </c>
       <c r="D7">
-        <v>3060</v>
+        <v>3037</v>
       </c>
       <c r="E7">
-        <v>0.99609375</v>
+        <v>0.9886067708333334</v>
       </c>
       <c r="F7">
         <v>0.9959038628472223</v>
       </c>
       <c r="G7">
-        <v>4.957126307985793</v>
+        <v>4.956801614236591</v>
       </c>
       <c r="H7">
         <v>5</v>
@@ -1210,10 +1231,10 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>0.03856209150326798</v>
+        <v>0.0388541323674679</v>
       </c>
       <c r="L7">
-        <v>0.01339869281045752</v>
+        <v>0.0135001646361541</v>
       </c>
       <c r="M7">
         <v>0</v>
@@ -1233,11 +1254,11 @@
       <c r="R7">
         <v>0.991742819843342</v>
       </c>
-      <c r="S7" t="b">
-        <v>1</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
+      <c r="S7">
+        <v>0.991742819843342</v>
+      </c>
+      <c r="T7" t="b">
+        <v>1</v>
       </c>
       <c r="U7">
         <v>0</v>
@@ -1249,48 +1270,51 @@
         <v>0</v>
       </c>
       <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
         <v>0.0009765625</v>
       </c>
-      <c r="Y7">
+      <c r="Z7">
         <v>0.01529947916666667</v>
       </c>
-      <c r="Z7">
-        <v>0</v>
-      </c>
       <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
         <v>0.01529947916666667</v>
       </c>
-      <c r="AB7">
+      <c r="AC7">
         <v>0.001302083333333333</v>
       </c>
-      <c r="AC7">
+      <c r="AD7">
         <v>0.0009765625</v>
       </c>
-      <c r="AD7">
-        <v>0</v>
-      </c>
       <c r="AE7">
         <v>0</v>
       </c>
       <c r="AF7">
-        <v>0.05196078431372549</v>
+        <v>0</v>
       </c>
       <c r="AG7">
-        <v>0.0009803921568627451</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>51</v>
+        <v>0.05235429700362199</v>
+      </c>
+      <c r="AH7">
+        <v>0.0009878169245966415</v>
       </c>
       <c r="AI7" t="s">
-        <v>54</v>
+        <v>52</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:35">
+    <row r="8" spans="1:36">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C8">
         <v>3072</v>
@@ -1340,10 +1364,10 @@
       <c r="R8">
         <v>0.991742796988247</v>
       </c>
-      <c r="S8" t="b">
-        <v>0</v>
-      </c>
-      <c r="T8">
+      <c r="S8">
+        <v>1</v>
+      </c>
+      <c r="T8" t="b">
         <v>0</v>
       </c>
       <c r="U8">
@@ -1356,48 +1380,51 @@
         <v>0</v>
       </c>
       <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
         <v>0.263671875</v>
       </c>
-      <c r="Y8">
+      <c r="Z8">
         <v>0.7509765625</v>
       </c>
-      <c r="Z8">
-        <v>0</v>
-      </c>
       <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
         <v>0.7509765625</v>
       </c>
-      <c r="AB8">
+      <c r="AC8">
         <v>0.3746744791666667</v>
       </c>
-      <c r="AC8">
+      <c r="AD8">
         <v>0.06966145833333333</v>
       </c>
-      <c r="AD8">
-        <v>0</v>
-      </c>
       <c r="AE8">
         <v>0</v>
       </c>
       <c r="AF8">
+        <v>0</v>
+      </c>
+      <c r="AG8">
         <v>0.753921568627451</v>
       </c>
-      <c r="AG8">
+      <c r="AH8">
         <v>0.06993464052287582</v>
       </c>
-      <c r="AH8" t="s">
-        <v>52</v>
-      </c>
       <c r="AI8" t="s">
-        <v>54</v>
+        <v>53</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>55</v>
       </c>
     </row>
-    <row r="9" spans="1:35">
+    <row r="9" spans="1:36">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C9">
         <v>3072</v>
@@ -1444,64 +1471,67 @@
       <c r="R9">
         <v>0</v>
       </c>
-      <c r="S9" t="b">
-        <v>0</v>
-      </c>
-      <c r="T9">
-        <v>0.001627604166666667</v>
+      <c r="S9">
+        <v>1</v>
+      </c>
+      <c r="T9" t="b">
+        <v>0</v>
       </c>
       <c r="U9">
         <v>0.001627604166666667</v>
       </c>
       <c r="V9">
-        <v>0</v>
+        <v>0.001627604166666667</v>
       </c>
       <c r="W9">
         <v>0</v>
       </c>
       <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
         <v>0.01009114583333333</v>
       </c>
-      <c r="Y9">
+      <c r="Z9">
         <v>0.02864583333333333</v>
       </c>
-      <c r="Z9">
-        <v>0</v>
-      </c>
       <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
         <v>0.02864583333333333</v>
       </c>
-      <c r="AB9">
+      <c r="AC9">
         <v>0.06673177083333333</v>
       </c>
-      <c r="AC9">
+      <c r="AD9">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AD9">
-        <v>0</v>
-      </c>
       <c r="AE9">
         <v>0</v>
       </c>
       <c r="AF9">
+        <v>0</v>
+      </c>
+      <c r="AG9">
         <v>0.02875816993464052</v>
       </c>
-      <c r="AG9">
+      <c r="AH9">
         <v>0.000326797385620915</v>
       </c>
-      <c r="AH9" t="s">
+      <c r="AI9" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:36">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
         <v>51</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="10" spans="1:35">
-      <c r="A10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B10" t="s">
-        <v>50</v>
       </c>
       <c r="C10">
         <v>3072</v>
@@ -1551,11 +1581,11 @@
       <c r="R10">
         <v>1</v>
       </c>
-      <c r="S10" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
+      <c r="S10">
+        <v>1</v>
+      </c>
+      <c r="T10" t="b">
+        <v>1</v>
       </c>
       <c r="U10">
         <v>0</v>
@@ -1567,20 +1597,20 @@
         <v>0</v>
       </c>
       <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
         <v>0.0006510416666666666</v>
       </c>
-      <c r="Y10">
+      <c r="Z10">
         <v>0.0009765625</v>
       </c>
-      <c r="Z10">
-        <v>0</v>
-      </c>
       <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
         <v>0.0009765625</v>
       </c>
-      <c r="AB10">
-        <v>0</v>
-      </c>
       <c r="AC10">
         <v>0</v>
       </c>
@@ -1591,24 +1621,27 @@
         <v>0</v>
       </c>
       <c r="AF10">
+        <v>0</v>
+      </c>
+      <c r="AG10">
         <v>0.0009803921568627451</v>
       </c>
-      <c r="AG10">
-        <v>0</v>
-      </c>
-      <c r="AH10" t="s">
+      <c r="AH10">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:36">
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" t="s">
         <v>51</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="11" spans="1:35">
-      <c r="A11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" t="s">
-        <v>50</v>
       </c>
       <c r="C11">
         <v>3072</v>
@@ -1658,15 +1691,15 @@
       <c r="R11">
         <v>1</v>
       </c>
-      <c r="S11" t="b">
-        <v>1</v>
-      </c>
-      <c r="T11">
+      <c r="S11">
+        <v>1</v>
+      </c>
+      <c r="T11" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11">
         <v>0.02278645833333333</v>
       </c>
-      <c r="U11">
-        <v>0</v>
-      </c>
       <c r="V11">
         <v>0</v>
       </c>
@@ -1677,17 +1710,17 @@
         <v>0</v>
       </c>
       <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
         <v>0.01009114583333333</v>
       </c>
-      <c r="Z11">
-        <v>0</v>
-      </c>
       <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
         <v>0.01009114583333333</v>
       </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
       <c r="AC11">
         <v>0</v>
       </c>
@@ -1698,24 +1731,27 @@
         <v>0</v>
       </c>
       <c r="AF11">
+        <v>0</v>
+      </c>
+      <c r="AG11">
         <v>0.03169934640522876</v>
       </c>
-      <c r="AG11">
-        <v>0</v>
-      </c>
-      <c r="AH11" t="s">
+      <c r="AH11">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:36">
+      <c r="A12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" t="s">
         <v>51</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="12" spans="1:35">
-      <c r="A12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" t="s">
-        <v>50</v>
       </c>
       <c r="C12">
         <v>3072</v>
@@ -1765,15 +1801,15 @@
       <c r="R12">
         <v>1</v>
       </c>
-      <c r="S12" t="b">
-        <v>1</v>
-      </c>
-      <c r="T12">
+      <c r="S12">
+        <v>1</v>
+      </c>
+      <c r="T12" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12">
         <v>0.1848958333333333</v>
       </c>
-      <c r="U12">
-        <v>0</v>
-      </c>
       <c r="V12">
         <v>0</v>
       </c>
@@ -1781,48 +1817,51 @@
         <v>0</v>
       </c>
       <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12">
         <v>0.06315104166666667</v>
       </c>
-      <c r="Y12">
+      <c r="Z12">
         <v>0.2298177083333333</v>
       </c>
-      <c r="Z12">
-        <v>0</v>
-      </c>
       <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
         <v>0.2298177083333333</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
         <v>0.01106770833333333</v>
       </c>
-      <c r="AC12">
+      <c r="AD12">
         <v>0.008138020833333334</v>
       </c>
-      <c r="AD12">
+      <c r="AE12">
         <v>0.008823529411764706</v>
       </c>
-      <c r="AE12">
-        <v>0</v>
-      </c>
       <c r="AF12">
+        <v>0</v>
+      </c>
+      <c r="AG12">
         <v>0.369281045751634</v>
       </c>
-      <c r="AG12">
+      <c r="AH12">
         <v>0.008169934640522876</v>
       </c>
-      <c r="AH12" t="s">
+      <c r="AI12" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" t="s">
         <v>51</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:35">
-      <c r="A13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" t="s">
-        <v>50</v>
       </c>
       <c r="C13">
         <v>3072</v>
@@ -1872,11 +1911,11 @@
       <c r="R13">
         <v>1</v>
       </c>
-      <c r="S13" t="b">
-        <v>1</v>
-      </c>
-      <c r="T13">
-        <v>0</v>
+      <c r="S13">
+        <v>1</v>
+      </c>
+      <c r="T13" t="b">
+        <v>1</v>
       </c>
       <c r="U13">
         <v>0</v>
@@ -1888,20 +1927,20 @@
         <v>0</v>
       </c>
       <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
         <v>0.0009765625</v>
       </c>
-      <c r="Y13">
+      <c r="Z13">
         <v>0.003255208333333333</v>
       </c>
-      <c r="Z13">
-        <v>0</v>
-      </c>
       <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
         <v>0.003255208333333333</v>
       </c>
-      <c r="AB13">
-        <v>0</v>
-      </c>
       <c r="AC13">
         <v>0</v>
       </c>
@@ -1912,24 +1951,27 @@
         <v>0</v>
       </c>
       <c r="AF13">
+        <v>0</v>
+      </c>
+      <c r="AG13">
         <v>0.00326797385620915</v>
       </c>
-      <c r="AG13">
-        <v>0</v>
-      </c>
-      <c r="AH13" t="s">
+      <c r="AH13">
+        <v>0</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
         <v>51</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:35">
-      <c r="A14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
       </c>
       <c r="C14">
         <v>3072</v>
@@ -1979,15 +2021,15 @@
       <c r="R14">
         <v>1</v>
       </c>
-      <c r="S14" t="b">
-        <v>1</v>
-      </c>
-      <c r="T14">
+      <c r="S14">
+        <v>1</v>
+      </c>
+      <c r="T14" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14">
         <v>0.002604166666666667</v>
       </c>
-      <c r="U14">
-        <v>0</v>
-      </c>
       <c r="V14">
         <v>0</v>
       </c>
@@ -2007,11 +2049,11 @@
         <v>0</v>
       </c>
       <c r="AB14">
+        <v>0</v>
+      </c>
+      <c r="AC14">
         <v>0.0003255208333333333</v>
       </c>
-      <c r="AC14">
-        <v>0</v>
-      </c>
       <c r="AD14">
         <v>0</v>
       </c>
@@ -2019,24 +2061,27 @@
         <v>0</v>
       </c>
       <c r="AF14">
+        <v>0</v>
+      </c>
+      <c r="AG14">
         <v>0.00261437908496732</v>
       </c>
-      <c r="AG14">
-        <v>0</v>
-      </c>
-      <c r="AH14" t="s">
+      <c r="AH14">
+        <v>0</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>52</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36">
+      <c r="A15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" t="s">
         <v>51</v>
-      </c>
-      <c r="AI14" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:35">
-      <c r="A15" t="s">
-        <v>48</v>
-      </c>
-      <c r="B15" t="s">
-        <v>50</v>
       </c>
       <c r="C15">
         <v>3072</v>
@@ -2086,15 +2131,15 @@
       <c r="R15">
         <v>1</v>
       </c>
-      <c r="S15" t="b">
-        <v>1</v>
-      </c>
-      <c r="T15">
+      <c r="S15">
+        <v>1</v>
+      </c>
+      <c r="T15" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15">
         <v>0.7119140625</v>
       </c>
-      <c r="U15">
-        <v>0</v>
-      </c>
       <c r="V15">
         <v>0</v>
       </c>
@@ -2102,40 +2147,43 @@
         <v>0</v>
       </c>
       <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
         <v>0.1103515625</v>
       </c>
-      <c r="Y15">
+      <c r="Z15">
         <v>0.2242838541666667</v>
       </c>
-      <c r="Z15">
-        <v>0</v>
-      </c>
       <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
         <v>0.2242838541666667</v>
       </c>
-      <c r="AB15">
+      <c r="AC15">
         <v>0.1373697916666667</v>
       </c>
-      <c r="AC15">
+      <c r="AD15">
         <v>0.01204427083333333</v>
       </c>
-      <c r="AD15">
-        <v>0</v>
-      </c>
       <c r="AE15">
         <v>0</v>
       </c>
       <c r="AF15">
+        <v>0</v>
+      </c>
+      <c r="AG15">
         <v>0.8320261437908497</v>
       </c>
-      <c r="AG15">
+      <c r="AH15">
         <v>0.01209150326797386</v>
-      </c>
-      <c r="AH15" t="s">
-        <v>53</v>
       </c>
       <c r="AI15" t="s">
         <v>54</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>